<commit_message>
cap nhat nut dang sua - 23072026
</commit_message>
<xml_diff>
--- a/Lịch sử sửa chữa nút THGT Huế.xlsx
+++ b/Lịch sử sửa chữa nút THGT Huế.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\THANGNM\1.SITECH\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\THANGNM\1.SITECH\19.THGT\1.HUE\sua_loi_nut_THGT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A99B2B09-1D32-478A-8CF8-3BDE65C18F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23EFA533-6F43-4F29-9873-6472B7BA2EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="795" yWindow="1950" windowWidth="24855" windowHeight="13530" activeTab="1" xr2:uid="{40324281-C953-4FDD-96A7-3374E4EAD2B1}"/>
+    <workbookView xWindow="2460" yWindow="1950" windowWidth="24855" windowHeight="13530" activeTab="2" xr2:uid="{40324281-C953-4FDD-96A7-3374E4EAD2B1}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="12-11-2025" sheetId="1" r:id="rId1"/>
     <sheet name="28-05-2026" sheetId="2" r:id="rId2"/>
+    <sheet name="23-07-2026" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="46">
   <si>
     <t>Ngày Nhận</t>
   </si>
@@ -157,13 +158,31 @@
   </si>
   <si>
     <t>Thay CM4</t>
+  </si>
+  <si>
+    <t>Bến Nghé - Đội Cung</t>
+  </si>
+  <si>
+    <t>Bình thường</t>
+  </si>
+  <si>
+    <t>Lê Duẩn - Yết Kêu</t>
+  </si>
+  <si>
+    <t>Hết Sim</t>
+  </si>
+  <si>
+    <t>Nguyễn Huệ - Lý Thường Kiệt</t>
+  </si>
+  <si>
+    <t>Phạm Văn Đồng - Tùng Thiện Vương</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,6 +191,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
       <sz val="13"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -305,7 +331,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -320,6 +346,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -350,10 +382,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -709,11 +741,11 @@
       <c r="B2" s="3">
         <v>46002</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="12"/>
-      <c r="E2" s="13"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="15"/>
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -735,13 +767,13 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="17">
-        <v>1</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="10">
+      <c r="A4" s="19">
+        <v>1</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="12">
         <v>6</v>
       </c>
       <c r="D4" s="8" t="s">
@@ -755,9 +787,9 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="18"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="10"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="12"/>
       <c r="D5" s="8" t="s">
         <v>3</v>
       </c>
@@ -772,9 +804,9 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="18"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="10"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="12"/>
       <c r="D6" s="7" t="s">
         <v>4</v>
       </c>
@@ -789,9 +821,9 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="18"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="10"/>
+      <c r="A7" s="20"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="12"/>
       <c r="D7" s="7" t="s">
         <v>5</v>
       </c>
@@ -803,9 +835,9 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="18"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="10"/>
+      <c r="A8" s="20"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="12"/>
       <c r="D8" s="7" t="s">
         <v>6</v>
       </c>
@@ -817,9 +849,9 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="19"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="10"/>
+      <c r="A9" s="21"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="12"/>
       <c r="D9" s="9" t="s">
         <v>25</v>
       </c>
@@ -876,123 +908,218 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="C2" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="10" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="20">
-        <v>1</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="21" t="s">
+      <c r="A3" s="10">
+        <v>1</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="10" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="20">
+      <c r="A4" s="10">
         <v>2</v>
       </c>
-      <c r="B4" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="21" t="s">
+      <c r="B4" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="E4" s="10" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="20">
+      <c r="A5" s="10">
         <v>3</v>
       </c>
-      <c r="B5" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5" s="21" t="s">
+      <c r="B5" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="10" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="20">
+      <c r="A6" s="10">
         <v>4</v>
       </c>
-      <c r="B6" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="21" t="s">
+      <c r="B6" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="10" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="20">
+      <c r="A7" s="10">
         <v>5</v>
       </c>
-      <c r="B7" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" s="21" t="s">
+      <c r="B7" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="E7" s="10" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="20">
+      <c r="A8" s="10">
         <v>6</v>
       </c>
-      <c r="B8" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" s="21" t="s">
+      <c r="B8" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="10" t="s">
         <v>39</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05ACF8F0-63AF-4B51-9933-3461CB8CFBB2}">
+  <dimension ref="B2:F6"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="9.140625" style="1"/>
+    <col min="3" max="3" width="12.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="37.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B2" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="5">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F3" s="5"/>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="5">
+        <v>2</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F4" s="5"/>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="5">
+        <v>3</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="5"/>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="5">
+        <v>4</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
them thong tin gateway sua chua
</commit_message>
<xml_diff>
--- a/Lịch sử sửa chữa nút THGT Huế.xlsx
+++ b/Lịch sử sửa chữa nút THGT Huế.xlsx
@@ -352,6 +352,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -381,12 +387,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -741,11 +741,11 @@
       <c r="B2" s="3">
         <v>46002</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="17"/>
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -767,13 +767,13 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="19">
-        <v>1</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="12">
+      <c r="A4" s="21">
+        <v>1</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="14">
         <v>6</v>
       </c>
       <c r="D4" s="8" t="s">
@@ -787,9 +787,9 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="20"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="12"/>
+      <c r="A5" s="22"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="14"/>
       <c r="D5" s="8" t="s">
         <v>3</v>
       </c>
@@ -804,9 +804,9 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="20"/>
-      <c r="B6" s="17"/>
-      <c r="C6" s="12"/>
+      <c r="A6" s="22"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="14"/>
       <c r="D6" s="7" t="s">
         <v>4</v>
       </c>
@@ -821,9 +821,9 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="20"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="12"/>
+      <c r="A7" s="22"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="14"/>
       <c r="D7" s="7" t="s">
         <v>5</v>
       </c>
@@ -835,9 +835,9 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="20"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="12"/>
+      <c r="A8" s="22"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="14"/>
       <c r="D8" s="7" t="s">
         <v>6</v>
       </c>
@@ -849,9 +849,9 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="21"/>
-      <c r="B9" s="18"/>
-      <c r="C9" s="12"/>
+      <c r="A9" s="23"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="14"/>
       <c r="D9" s="9" t="s">
         <v>25</v>
       </c>
@@ -1045,19 +1045,19 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="22" t="s">
+      <c r="E2" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="12" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
       <c r="C3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="13" t="s">
         <v>40</v>
       </c>
       <c r="E3" s="5" t="s">
@@ -1083,7 +1083,7 @@
       <c r="C4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="13" t="s">
         <v>42</v>
       </c>
       <c r="E4" s="5" t="s">
@@ -1098,7 +1098,7 @@
       <c r="C5" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="13" t="s">
         <v>44</v>
       </c>
       <c r="E5" s="5" t="s">
@@ -1113,7 +1113,7 @@
       <c r="C6" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="D6" s="13" t="s">
         <v>45</v>
       </c>
       <c r="E6" s="5" t="s">

</xml_diff>